<commit_message>
updated aluminum frame baseline
Used Yuan et al 2024. need to add steel frame
</commit_message>
<xml_diff>
--- a/PV_ICE/baselines/SupportingMaterial/Manual Files/MaterialCompositionAnnual-Graph.xlsx
+++ b/PV_ICE/baselines/SupportingMaterial/Manual Files/MaterialCompositionAnnual-Graph.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hmirletz\Documents\GitHub\PV_ICE\PV_ICE\baselines\SupportingMaterial\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hmirletz\Documents\GitHub\PV_ICE\PV_ICE\baselines\SupportingMaterial\Manual Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1B87E4B-0985-49BF-97AE-1CC5244377F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47669CC1-64CE-4C46-B4CC-7868F55BAD2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0FB8D6CD-8546-4236-B63D-A974CB21DD58}"/>
+    <workbookView xWindow="-28920" yWindow="45" windowWidth="29040" windowHeight="15720" xr2:uid="{0FB8D6CD-8546-4236-B63D-A974CB21DD58}"/>
   </bookViews>
   <sheets>
     <sheet name="Silicon" sheetId="1" r:id="rId1"/>
@@ -858,7 +858,9 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="1F77BE"/>
+              <a:schemeClr val="bg1">
+                <a:lumMod val="50000"/>
+              </a:schemeClr>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1082,139 +1084,139 @@
                   <c:v>2113.8328529999999</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2083.4794809999999</c:v>
+                  <c:v>2438.13</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2054.6821599999998</c:v>
+                  <c:v>2686.73</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2027.3242250000001</c:v>
+                  <c:v>1826.82</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2001.3003900000001</c:v>
+                  <c:v>2250.65</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1987.1506589999999</c:v>
+                  <c:v>1885.12</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1966.59313</c:v>
+                  <c:v>1923.63</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1962.9861980000001</c:v>
+                  <c:v>1853.31</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1619.458128</c:v>
+                  <c:v>1641.14</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>1592.739726</c:v>
+                  <c:v>1839.32</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1495.242424</c:v>
+                  <c:v>1688.23</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>1412.526316</c:v>
+                  <c:v>1670.89</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1379.8208959999999</c:v>
+                  <c:v>1615.33</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>1361.666667</c:v>
+                  <c:v>1553.01</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1343.6470589999999</c:v>
+                  <c:v>1573.85</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1343.6470589999999</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>1272.176471</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>1250.7352940000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>1229.294118</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>1215</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>1200.705882</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>1191.176471</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>1181.6470589999999</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>1172.117647</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>1162.5882349999999</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>1153.058824</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>1143.5294120000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1241,10 +1243,12 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="FF7F0E"/>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:ln>
-              <a:noFill/>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
@@ -3550,7 +3554,9 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="1F77BE"/>
+              <a:schemeClr val="bg1">
+                <a:lumMod val="50000"/>
+              </a:schemeClr>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -3714,79 +3720,79 @@
                   <c:v>2113.8328529999999</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2083.4794809999999</c:v>
+                  <c:v>2438.13</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2054.6821599999998</c:v>
+                  <c:v>2686.73</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2027.3242250000001</c:v>
+                  <c:v>1826.82</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2001.3003900000001</c:v>
+                  <c:v>2250.65</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1987.1506589999999</c:v>
+                  <c:v>1885.12</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1966.59313</c:v>
+                  <c:v>1923.63</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1962.9861980000001</c:v>
+                  <c:v>1853.31</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1619.458128</c:v>
+                  <c:v>1641.14</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>1592.739726</c:v>
+                  <c:v>1839.32</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1495.242424</c:v>
+                  <c:v>1688.23</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>1412.526316</c:v>
+                  <c:v>1670.89</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1379.8208959999999</c:v>
+                  <c:v>1615.33</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>1361.666667</c:v>
+                  <c:v>1553.01</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1343.6470589999999</c:v>
+                  <c:v>1573.85</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1343.6470589999999</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>1272.176471</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>1250.7352940000001</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>1229.294118</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>1215</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>1200.705882</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>1191.176471</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>1181.6470589999999</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>1172.117647</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>1162.5882349999999</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>1153.058824</c:v>
+                  <c:v>1579.96</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3813,7 +3819,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="FF7F0E"/>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -4339,7 +4345,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="2CA02C"/>
+              <a:schemeClr val="accent4"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -13093,7 +13099,7 @@
         <v>8000</v>
       </c>
       <c r="C13">
-        <v>2083.4794809999999</v>
+        <v>2438.13</v>
       </c>
       <c r="D13">
         <v>465.8</v>
@@ -13112,39 +13118,39 @@
       </c>
       <c r="I13">
         <f t="shared" si="1"/>
-        <v>11703.680709439999</v>
+        <v>12058.33122844</v>
       </c>
       <c r="J13">
         <f t="shared" si="2"/>
-        <v>11.703680709439999</v>
+        <v>12.05833122844</v>
       </c>
       <c r="L13" s="1">
         <f t="shared" si="3"/>
-        <v>68.354564675942754</v>
+        <v>66.344171912708106</v>
       </c>
       <c r="M13" s="1">
         <f t="shared" si="4"/>
-        <v>17.801916616876767</v>
+        <v>20.219464483191377</v>
       </c>
       <c r="N13" s="1">
         <f t="shared" si="5"/>
-        <v>3.9799445282567665</v>
+        <v>3.8628894096174293</v>
       </c>
       <c r="O13" s="1">
         <f t="shared" si="6"/>
-        <v>0.27498064872909456</v>
+        <v>0.26689312584228569</v>
       </c>
       <c r="P13" s="1">
         <f t="shared" si="7"/>
-        <v>4.593426746223353E-2</v>
+        <v>4.4583283525339849E-2</v>
       </c>
       <c r="Q13" s="1">
         <f t="shared" si="8"/>
-        <v>7.2284952144809456</v>
+        <v>7.0158961797688812</v>
       </c>
       <c r="R13" s="1">
         <f t="shared" si="9"/>
-        <v>2.3141640482514445</v>
+        <v>2.2461016053465901</v>
       </c>
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.35">
@@ -13155,7 +13161,7 @@
         <v>8000</v>
       </c>
       <c r="C14">
-        <v>2054.6821599999998</v>
+        <v>2686.73</v>
       </c>
       <c r="D14">
         <v>442.51</v>
@@ -13174,39 +13180,39 @@
       </c>
       <c r="I14">
         <f t="shared" si="1"/>
-        <v>11675.947875330001</v>
+        <v>12307.99571533</v>
       </c>
       <c r="J14">
         <f t="shared" si="2"/>
-        <v>11.675947875330001</v>
+        <v>12.30799571533</v>
       </c>
       <c r="L14" s="1">
         <f t="shared" si="3"/>
-        <v>68.516921156381002</v>
+        <v>64.99839766791392</v>
       </c>
       <c r="M14" s="1">
         <f t="shared" si="4"/>
-        <v>17.597561944767826</v>
+        <v>21.829143120789297</v>
       </c>
       <c r="N14" s="1">
         <f t="shared" si="5"/>
-        <v>3.7899278476137699</v>
+        <v>3.5953051190035739</v>
       </c>
       <c r="O14" s="1">
         <f t="shared" si="6"/>
-        <v>0.25684057303272623</v>
+        <v>0.24365113641247274</v>
       </c>
       <c r="P14" s="1">
         <f t="shared" si="7"/>
-        <v>4.6043371017088039E-2</v>
+        <v>4.3678923232838153E-2</v>
       </c>
       <c r="Q14" s="1">
         <f t="shared" si="8"/>
-        <v>7.245664412287292</v>
+        <v>6.8735805533818972</v>
       </c>
       <c r="R14" s="1">
         <f t="shared" si="9"/>
-        <v>2.5470406949002822</v>
+        <v>2.4162434792660012</v>
       </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.35">
@@ -13217,7 +13223,7 @@
         <v>8000</v>
       </c>
       <c r="C15">
-        <v>2027.3242250000001</v>
+        <v>1826.82</v>
       </c>
       <c r="D15">
         <v>419.22</v>
@@ -13236,39 +13242,39 @@
       </c>
       <c r="I15">
         <f t="shared" si="1"/>
-        <v>11649.58719591</v>
+        <v>11449.08297091</v>
       </c>
       <c r="J15">
         <f t="shared" si="2"/>
-        <v>11.64958719591</v>
+        <v>11.44908297091</v>
       </c>
       <c r="L15" s="1">
         <f t="shared" si="3"/>
-        <v>68.671961207421006</v>
+        <v>69.874591880646847</v>
       </c>
       <c r="M15" s="1">
         <f t="shared" si="4"/>
-        <v>17.402541316758107</v>
+        <v>15.95603774242541</v>
       </c>
       <c r="N15" s="1">
         <f t="shared" si="5"/>
-        <v>3.5985824471718795</v>
+        <v>3.6616033010255968</v>
       </c>
       <c r="O15" s="1">
         <f t="shared" si="6"/>
-        <v>0.23858601375813698</v>
+        <v>0.24276429632504309</v>
       </c>
       <c r="P15" s="1">
         <f t="shared" si="7"/>
-        <v>4.6147557931386918E-2</v>
+        <v>4.6955725743794689E-2</v>
       </c>
       <c r="Q15" s="1">
         <f t="shared" si="8"/>
-        <v>7.2620598976847708</v>
+        <v>7.3892380913784041</v>
       </c>
       <c r="R15" s="1">
         <f t="shared" si="9"/>
-        <v>2.7801215592747091</v>
+        <v>2.8288089624549015</v>
       </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.35">
@@ -13279,7 +13285,7 @@
         <v>8000</v>
       </c>
       <c r="C16">
-        <v>2001.3003900000001</v>
+        <v>2250.65</v>
       </c>
       <c r="D16">
         <v>419.22</v>
@@ -13298,39 +13304,39 @@
       </c>
       <c r="I16">
         <f t="shared" si="1"/>
-        <v>11647.782635400001</v>
+        <v>11897.1322454</v>
       </c>
       <c r="J16">
         <f t="shared" si="2"/>
-        <v>11.6477826354</v>
+        <v>11.8971322454</v>
       </c>
       <c r="L16" s="1">
         <f t="shared" si="3"/>
-        <v>68.682600374824645</v>
+        <v>67.243095520714107</v>
       </c>
       <c r="M16" s="1">
         <f t="shared" si="4"/>
-        <v>17.181814364543836</v>
+        <v>18.9175841167119</v>
       </c>
       <c r="N16" s="1">
         <f t="shared" si="5"/>
-        <v>3.5991399661417485</v>
+        <v>3.5237063130242205</v>
       </c>
       <c r="O16" s="1">
         <f t="shared" si="6"/>
-        <v>0.21978432119943886</v>
+        <v>0.21517790566628514</v>
       </c>
       <c r="P16" s="1">
         <f t="shared" si="7"/>
-        <v>4.615470745188216E-2</v>
+        <v>4.5187360189919874E-2</v>
       </c>
       <c r="Q16" s="1">
         <f t="shared" si="8"/>
-        <v>7.2631849896377059</v>
+        <v>7.1109573513155153</v>
       </c>
       <c r="R16" s="1">
         <f t="shared" si="9"/>
-        <v>3.0073212762007442</v>
+        <v>2.944291432378062</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.35">
@@ -13341,7 +13347,7 @@
         <v>8000</v>
       </c>
       <c r="C17">
-        <v>1987.1506589999999</v>
+        <v>1885.12</v>
       </c>
       <c r="D17">
         <v>419.22</v>
@@ -13360,39 +13366,39 @@
       </c>
       <c r="I17">
         <f t="shared" si="1"/>
-        <v>11646.705138569998</v>
+        <v>11544.674479569998</v>
       </c>
       <c r="J17">
         <f t="shared" si="2"/>
-        <v>11.646705138569997</v>
+        <v>11.544674479569998</v>
       </c>
       <c r="L17" s="1">
         <f t="shared" si="3"/>
-        <v>68.68895455682717</v>
+        <v>69.296020551789297</v>
       </c>
       <c r="M17" s="1">
         <f t="shared" si="4"/>
-        <v>17.06191266420252</v>
+        <v>16.328914282823629</v>
       </c>
       <c r="N17" s="1">
         <f t="shared" si="5"/>
-        <v>3.5994729411641355</v>
+        <v>3.6312847169651392</v>
       </c>
       <c r="O17" s="1">
         <f t="shared" si="6"/>
-        <v>0.1058446661380283</v>
+        <v>0.10678011053334745</v>
       </c>
       <c r="P17" s="1">
         <f t="shared" si="7"/>
-        <v>4.6158977462187854E-2</v>
+        <v>4.6566925810802406E-2</v>
       </c>
       <c r="Q17" s="1">
         <f t="shared" si="8"/>
-        <v>7.2638569443844725</v>
+        <v>7.3280541733517186</v>
       </c>
       <c r="R17" s="1">
         <f t="shared" si="9"/>
-        <v>3.2337992498215118</v>
+        <v>3.2623792387260826</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.35">
@@ -13403,7 +13409,7 @@
         <v>8000</v>
       </c>
       <c r="C18">
-        <v>1966.59313</v>
+        <v>1923.63</v>
       </c>
       <c r="D18">
         <v>419.22</v>
@@ -13422,39 +13428,39 @@
       </c>
       <c r="I18">
         <f t="shared" si="1"/>
-        <v>11650.368343809998</v>
+        <v>11607.40521381</v>
       </c>
       <c r="J18">
         <f t="shared" si="2"/>
-        <v>11.650368343809998</v>
+        <v>11.607405213809999</v>
       </c>
       <c r="L18" s="1">
         <f t="shared" si="3"/>
-        <v>68.667356807224991</v>
+        <v>68.921519087504052</v>
       </c>
       <c r="M18" s="1">
         <f t="shared" si="4"/>
-        <v>16.880094019043426</v>
+        <v>16.572437720286928</v>
       </c>
       <c r="N18" s="1">
         <f t="shared" si="5"/>
-        <v>3.5983411650906079</v>
+        <v>3.6116599039829311</v>
       </c>
       <c r="O18" s="1">
         <f t="shared" si="6"/>
-        <v>8.8176154666029141E-2</v>
+        <v>8.8502525937302526E-2</v>
       </c>
       <c r="P18" s="1">
         <f t="shared" si="7"/>
-        <v>4.6144463774455198E-2</v>
+        <v>4.6315260826802727E-2</v>
       </c>
       <c r="Q18" s="1">
         <f t="shared" si="8"/>
-        <v>7.2615729823640427</v>
+        <v>7.2884506435035536</v>
       </c>
       <c r="R18" s="1">
         <f t="shared" si="9"/>
-        <v>3.4583144078364674</v>
+        <v>3.4711148579584266</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.35">
@@ -13465,7 +13471,7 @@
         <v>8045</v>
       </c>
       <c r="C19">
-        <v>1962.9861980000001</v>
+        <v>1853.31</v>
       </c>
       <c r="D19">
         <v>419.22</v>
@@ -13484,39 +13490,39 @@
       </c>
       <c r="I19">
         <f t="shared" si="1"/>
-        <v>11711.620733948999</v>
+        <v>11601.944535948998</v>
       </c>
       <c r="J19">
         <f t="shared" si="2"/>
-        <v>11.711620733948999</v>
+        <v>11.601944535948999</v>
       </c>
       <c r="L19" s="1">
         <f t="shared" si="3"/>
-        <v>68.692456686883645</v>
+        <v>69.34182433877622</v>
       </c>
       <c r="M19" s="1">
         <f t="shared" si="4"/>
-        <v>16.761012353395323</v>
+        <v>15.974132562498117</v>
       </c>
       <c r="N19" s="1">
         <f t="shared" si="5"/>
-        <v>3.5795216522405671</v>
+        <v>3.6133598010319163</v>
       </c>
       <c r="O19" s="1">
         <f t="shared" si="6"/>
-        <v>7.0171991013825361E-2</v>
+        <v>7.0835345088363449E-2</v>
       </c>
       <c r="P19" s="1">
         <f t="shared" si="7"/>
-        <v>4.5903125810899496E-2</v>
+        <v>4.6337059993195893E-2</v>
       </c>
       <c r="Q19" s="1">
         <f t="shared" si="8"/>
-        <v>7.2235945751527115</v>
+        <v>7.2918810926792643</v>
       </c>
       <c r="R19" s="1">
         <f t="shared" si="9"/>
-        <v>3.6273396155030406</v>
+        <v>3.6616297999329404</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.35">
@@ -13527,7 +13533,7 @@
         <v>8090</v>
       </c>
       <c r="C20">
-        <v>1619.458128</v>
+        <v>1641.14</v>
       </c>
       <c r="D20">
         <v>419.22</v>
@@ -13546,39 +13552,39 @@
       </c>
       <c r="I20">
         <f t="shared" si="1"/>
-        <v>11431.947299613999</v>
+        <v>11453.629171613999</v>
       </c>
       <c r="J20">
         <f t="shared" si="2"/>
-        <v>11.431947299613999</v>
+        <v>11.453629171613999</v>
       </c>
       <c r="L20" s="1">
         <f t="shared" si="3"/>
-        <v>70.766596345953758</v>
+        <v>70.632634240069351</v>
       </c>
       <c r="M20" s="1">
         <f t="shared" si="4"/>
-        <v>14.166074121551286</v>
+        <v>14.328558882169027</v>
       </c>
       <c r="N20" s="1">
         <f t="shared" si="5"/>
-        <v>3.6670917824660982</v>
+        <v>3.6601499290632722</v>
       </c>
       <c r="O20" s="1">
         <f t="shared" si="6"/>
-        <v>5.0322084796474202E-2</v>
+        <v>5.0226824422231052E-2</v>
       </c>
       <c r="P20" s="1">
         <f t="shared" si="7"/>
-        <v>4.702610901802811E-2</v>
+        <v>4.6937087969667841E-2</v>
       </c>
       <c r="Q20" s="1">
         <f t="shared" si="8"/>
-        <v>7.4003140307387989</v>
+        <v>7.3863051380838902</v>
       </c>
       <c r="R20" s="1">
         <f t="shared" si="9"/>
-        <v>3.9025755254755587</v>
+        <v>3.8951878982225829</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.35">
@@ -13589,7 +13595,7 @@
         <v>8180</v>
       </c>
       <c r="C21">
-        <v>1592.739726</v>
+        <v>1839.32</v>
       </c>
       <c r="D21">
         <v>419.22</v>
@@ -13608,39 +13614,39 @@
       </c>
       <c r="I21">
         <f t="shared" si="1"/>
-        <v>11500.887606342001</v>
+        <v>11747.467880342001</v>
       </c>
       <c r="J21">
         <f t="shared" si="2"/>
-        <v>11.500887606342001</v>
+        <v>11.747467880342001</v>
       </c>
       <c r="L21" s="1">
         <f t="shared" si="3"/>
-        <v>71.124945134575995</v>
+        <v>69.63202694674537</v>
       </c>
       <c r="M21" s="1">
         <f t="shared" si="4"/>
-        <v>13.848841763497507</v>
+        <v>15.657161345194096</v>
       </c>
       <c r="N21" s="1">
         <f t="shared" si="5"/>
-        <v>3.6451099632416812</v>
+        <v>3.5685988186570414</v>
       </c>
       <c r="O21" s="1">
         <f t="shared" si="6"/>
-        <v>4.6447548440124706E-2</v>
+        <v>4.547261074821924E-2</v>
       </c>
       <c r="P21" s="1">
         <f t="shared" si="7"/>
-        <v>4.6744218220474407E-2</v>
+        <v>4.5763053406565175E-2</v>
       </c>
       <c r="Q21" s="1">
         <f t="shared" si="8"/>
-        <v>7.3741264937875997</v>
+        <v>7.2193429991766855</v>
       </c>
       <c r="R21" s="1">
         <f t="shared" si="9"/>
-        <v>3.9137848782365952</v>
+        <v>3.831634226072008</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.35">
@@ -13651,7 +13657,7 @@
         <v>8090</v>
       </c>
       <c r="C22">
-        <v>1495.242424</v>
+        <v>1688.23</v>
       </c>
       <c r="D22">
         <v>419.22</v>
@@ -13670,39 +13676,39 @@
       </c>
       <c r="I22">
         <f t="shared" si="1"/>
-        <v>11334.099356297</v>
+        <v>11527.086932296999</v>
       </c>
       <c r="J22">
         <f t="shared" si="2"/>
-        <v>11.334099356296999</v>
+        <v>11.527086932296999</v>
       </c>
       <c r="L22" s="1">
         <f t="shared" si="3"/>
-        <v>71.37752851535889</v>
+        <v>70.18251920468434</v>
       </c>
       <c r="M22" s="1">
         <f t="shared" si="4"/>
-        <v>13.192423826506101</v>
+        <v>14.645764449558001</v>
       </c>
       <c r="N22" s="1">
         <f t="shared" si="5"/>
-        <v>3.6987500005202421</v>
+        <v>3.6368251793557196</v>
       </c>
       <c r="O22" s="1">
         <f t="shared" si="6"/>
-        <v>3.9880121524510453E-2</v>
+        <v>3.9212444770721361E-2</v>
       </c>
       <c r="P22" s="1">
         <f t="shared" si="7"/>
-        <v>5.1068548263468447E-2</v>
+        <v>5.0213553814559421E-2</v>
       </c>
       <c r="Q22" s="1">
         <f t="shared" si="8"/>
-        <v>7.501963528558635</v>
+        <v>7.3763649480048192</v>
       </c>
       <c r="R22" s="1">
         <f t="shared" si="9"/>
-        <v>4.1383854592681502</v>
+        <v>4.0691002198118476</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.35">
@@ -13713,7 +13719,7 @@
         <v>8135</v>
       </c>
       <c r="C23">
-        <v>1412.526316</v>
+        <v>1670.89</v>
       </c>
       <c r="D23">
         <v>419.22</v>
@@ -13732,39 +13738,39 @@
       </c>
       <c r="I23">
         <f t="shared" si="1"/>
-        <v>11318.409426708999</v>
+        <v>11576.773110708999</v>
       </c>
       <c r="J23">
         <f t="shared" si="2"/>
-        <v>11.318409426708998</v>
+        <v>11.576773110708999</v>
       </c>
       <c r="L23" s="1">
         <f t="shared" si="3"/>
-        <v>71.874056621446826</v>
+        <v>70.270013260213119</v>
       </c>
       <c r="M23" s="1">
         <f t="shared" si="4"/>
-        <v>12.479901218865111</v>
+        <v>14.433123842207438</v>
       </c>
       <c r="N23" s="1">
         <f t="shared" si="5"/>
-        <v>3.7038773222916945</v>
+        <v>3.6212163440622676</v>
       </c>
       <c r="O23" s="1">
         <f t="shared" si="6"/>
-        <v>3.622202426540129E-2</v>
+        <v>3.5413642210950419E-2</v>
       </c>
       <c r="P23" s="1">
         <f t="shared" si="7"/>
-        <v>5.478084213289356E-2</v>
+        <v>5.3558275183474433E-2</v>
       </c>
       <c r="Q23" s="1">
         <f t="shared" si="8"/>
-        <v>7.5347159468145133</v>
+        <v>7.3665605419105527</v>
       </c>
       <c r="R23" s="1">
         <f t="shared" si="9"/>
-        <v>4.3164460241835787</v>
+        <v>4.220114094212212</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.35">
@@ -13775,7 +13781,7 @@
         <v>8208.375</v>
       </c>
       <c r="C24">
-        <v>1379.8208959999999</v>
+        <v>1615.33</v>
       </c>
       <c r="D24">
         <v>419.22</v>
@@ -13794,39 +13800,39 @@
       </c>
       <c r="I24">
         <f t="shared" si="1"/>
-        <v>11347.112359453999</v>
+        <v>11582.621463453999</v>
       </c>
       <c r="J24">
         <f t="shared" si="2"/>
-        <v>11.347112359453998</v>
+        <v>11.582621463454</v>
       </c>
       <c r="L24" s="1">
         <f t="shared" si="3"/>
-        <v>72.338888873001096</v>
+        <v>70.868024357866048</v>
       </c>
       <c r="M24" s="1">
         <f t="shared" si="4"/>
-        <v>12.160106045397388</v>
+        <v>13.946152044222121</v>
       </c>
       <c r="N24" s="1">
         <f t="shared" si="5"/>
-        <v>3.6945082301112606</v>
+        <v>3.6193879021492807</v>
       </c>
       <c r="O24" s="1">
         <f t="shared" si="6"/>
-        <v>3.5953700155272876E-2</v>
+        <v>3.5222654619875747E-2</v>
       </c>
       <c r="P24" s="1">
         <f t="shared" si="7"/>
-        <v>6.3486107934747155E-2</v>
+        <v>6.2195246755925457E-2</v>
       </c>
       <c r="Q24" s="1">
         <f t="shared" si="8"/>
-        <v>7.4731788417824712</v>
+        <v>7.3212269146118221</v>
       </c>
       <c r="R24" s="1">
         <f t="shared" si="9"/>
-        <v>4.2338782016177818</v>
+        <v>4.1477908797749432</v>
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.35">
@@ -13837,7 +13843,7 @@
         <v>8253.5499999999993</v>
       </c>
       <c r="C25">
-        <v>1361.666667</v>
+        <v>1553.01</v>
       </c>
       <c r="D25">
         <v>410.85500830000001</v>
@@ -13856,39 +13862,39 @@
       </c>
       <c r="I25">
         <f t="shared" si="1"/>
-        <v>11359.694053671998</v>
+        <v>11551.037386671998</v>
       </c>
       <c r="J25">
         <f t="shared" si="2"/>
-        <v>11.359694053671998</v>
+        <v>11.551037386671998</v>
       </c>
       <c r="L25" s="1">
         <f t="shared" si="3"/>
-        <v>72.656446212405314</v>
+        <v>71.452889673123579</v>
       </c>
       <c r="M25" s="1">
         <f t="shared" si="4"/>
-        <v>11.986825178270044</v>
+        <v>13.444766457010335</v>
       </c>
       <c r="N25" s="1">
         <f t="shared" si="5"/>
-        <v>3.616778817799164</v>
+        <v>3.5568667518474082</v>
       </c>
       <c r="O25" s="1">
         <f t="shared" si="6"/>
-        <v>3.7979236514784513E-2</v>
+        <v>3.735010915104494E-2</v>
       </c>
       <c r="P25" s="1">
         <f t="shared" si="7"/>
-        <v>6.562430259809926E-2</v>
+        <v>6.4537233760506435E-2</v>
       </c>
       <c r="Q25" s="1">
         <f t="shared" si="8"/>
-        <v>7.4733966952708304</v>
+        <v>7.3495996210656793</v>
       </c>
       <c r="R25" s="1">
         <f t="shared" si="9"/>
-        <v>4.1629495571417836</v>
+        <v>4.0939901540414638</v>
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.35">
@@ -13899,7 +13905,7 @@
         <v>8450</v>
       </c>
       <c r="C26">
-        <v>1343.6470589999999</v>
+        <v>1573.85</v>
       </c>
       <c r="D26">
         <v>402.1406667</v>
@@ -13918,39 +13924,39 @@
       </c>
       <c r="I26">
         <f t="shared" si="1"/>
-        <v>11522.693239491997</v>
+        <v>11752.896180491998</v>
       </c>
       <c r="J26">
         <f t="shared" si="2"/>
-        <v>11.522693239491996</v>
+        <v>11.752896180491998</v>
       </c>
       <c r="L26" s="1">
         <f t="shared" si="3"/>
-        <v>73.333549929448054</v>
+        <v>71.897172154261867</v>
       </c>
       <c r="M26" s="1">
         <f t="shared" si="4"/>
-        <v>11.660876767897342</v>
+        <v>13.391167384021898</v>
       </c>
       <c r="N26" s="1">
         <f t="shared" si="5"/>
-        <v>3.4899884804859149</v>
+        <v>3.4216303839005375</v>
       </c>
       <c r="O26" s="1">
         <f t="shared" si="6"/>
-        <v>3.5776304257334753E-2</v>
+        <v>3.507555694095673E-2</v>
       </c>
       <c r="P26" s="1">
         <f t="shared" si="7"/>
-        <v>7.1694349821675982E-2</v>
+        <v>7.0290078914439738E-2</v>
       </c>
       <c r="Q26" s="1">
         <f t="shared" si="8"/>
-        <v>7.3881164959098733</v>
+        <v>7.2434061096620912</v>
       </c>
       <c r="R26" s="1">
         <f t="shared" si="9"/>
-        <v>4.0199976721798221</v>
+        <v>3.9412583322982191</v>
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.35">
@@ -13961,7 +13967,7 @@
         <v>8764.1</v>
       </c>
       <c r="C27">
-        <v>1343.6470589999999</v>
+        <v>1579.96</v>
       </c>
       <c r="D27">
         <v>395.54183339999997</v>
@@ -13980,39 +13986,39 @@
       </c>
       <c r="I27">
         <f t="shared" si="1"/>
-        <v>11796.884007142004</v>
+        <v>12033.196948142004</v>
       </c>
       <c r="J27">
         <f t="shared" si="2"/>
-        <v>11.796884007142003</v>
+        <v>12.033196948142004</v>
       </c>
       <c r="L27" s="1">
         <f t="shared" si="3"/>
-        <v>74.291651886159841</v>
+        <v>72.832681437606055</v>
       </c>
       <c r="M27" s="1">
         <f t="shared" si="4"/>
-        <v>11.38984716800247</v>
+        <v>13.130010310717594</v>
       </c>
       <c r="N27" s="1">
         <f t="shared" si="5"/>
-        <v>3.3529348356780759</v>
+        <v>3.2870885027862355</v>
       </c>
       <c r="O27" s="1">
         <f t="shared" si="6"/>
-        <v>2.8753650031198182E-2</v>
+        <v>2.8188973858054817E-2</v>
       </c>
       <c r="P27" s="1">
         <f t="shared" si="7"/>
-        <v>6.9724174578815024E-2</v>
+        <v>6.8354902154826203E-2</v>
       </c>
       <c r="Q27" s="1">
         <f t="shared" si="8"/>
-        <v>7.2005878796954663</v>
+        <v>7.0591797313776974</v>
       </c>
       <c r="R27" s="1">
         <f t="shared" si="9"/>
-        <v>3.6665004058541091</v>
+        <v>3.5944961414995009</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.35">
@@ -14023,7 +14029,7 @@
         <v>9076.6</v>
       </c>
       <c r="C28">
-        <v>1272.176471</v>
+        <v>1579.96</v>
       </c>
       <c r="D28">
         <v>388.94299999999998</v>
@@ -14042,39 +14048,39 @@
       </c>
       <c r="I28">
         <f t="shared" si="1"/>
-        <v>11968.022566373</v>
+        <v>12275.806095373</v>
       </c>
       <c r="J28">
         <f t="shared" si="2"/>
-        <v>11.968022566373</v>
+        <v>12.275806095372999</v>
       </c>
       <c r="L28" s="1">
         <f t="shared" si="3"/>
-        <v>75.840431864682998</v>
+        <v>73.938932641019434</v>
       </c>
       <c r="M28" s="1">
         <f t="shared" si="4"/>
-        <v>10.6297967266078</v>
+        <v>12.870519359176901</v>
       </c>
       <c r="N28" s="1">
         <f t="shared" si="5"/>
-        <v>3.2498518267573098</v>
+        <v>3.1683703455254189</v>
       </c>
       <c r="O28" s="1">
         <f t="shared" si="6"/>
-        <v>2.9303214909151262E-2</v>
+        <v>2.8568513918787501E-2</v>
       </c>
       <c r="P28" s="1">
         <f t="shared" si="7"/>
-        <v>6.9101473983152015E-2</v>
+        <v>6.7368936392023654E-2</v>
       </c>
       <c r="Q28" s="1">
         <f t="shared" si="8"/>
-        <v>6.7656122430373129</v>
+        <v>6.5959823225392595</v>
       </c>
       <c r="R28" s="1">
         <f t="shared" si="9"/>
-        <v>3.4159026500222818</v>
+        <v>3.330257881428178</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.35">
@@ -14085,7 +14091,7 @@
         <v>9484.2124999999996</v>
       </c>
       <c r="C29">
-        <v>1250.7352940000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D29">
         <v>384.28500000000003</v>
@@ -14104,39 +14110,39 @@
       </c>
       <c r="I29">
         <f t="shared" si="1"/>
-        <v>12311.858246171001</v>
+        <v>12641.082952171002</v>
       </c>
       <c r="J29">
         <f t="shared" si="2"/>
-        <v>12.311858246171001</v>
+        <v>12.641082952171002</v>
       </c>
       <c r="L29" s="1">
         <f t="shared" si="3"/>
-        <v>77.033152188456995</v>
+        <v>75.026898691232489</v>
       </c>
       <c r="M29" s="1">
         <f t="shared" si="4"/>
-        <v>10.158785692557659</v>
+        <v>12.49861270571486</v>
       </c>
       <c r="N29" s="1">
         <f t="shared" si="5"/>
-        <v>3.1212591334010282</v>
+        <v>3.0399689761865081</v>
       </c>
       <c r="O29" s="1">
         <f t="shared" si="6"/>
-        <v>2.6201342693360274E-2</v>
+        <v>2.5518954216228629E-2</v>
       </c>
       <c r="P29" s="1">
         <f t="shared" si="7"/>
-        <v>6.7535540401351971E-2</v>
+        <v>6.5776642962160042E-2</v>
       </c>
       <c r="Q29" s="1">
         <f t="shared" si="8"/>
-        <v>6.3573465869250292</v>
+        <v>6.1917756806237589</v>
       </c>
       <c r="R29" s="1">
         <f t="shared" si="9"/>
-        <v>3.2357195155645626</v>
+        <v>3.15144834906397</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.35">
@@ -14147,7 +14153,7 @@
         <v>9654.375</v>
       </c>
       <c r="C30">
-        <v>1229.294118</v>
+        <v>1579.96</v>
       </c>
       <c r="D30">
         <v>374.96899999999999</v>
@@ -14166,39 +14172,39 @@
       </c>
       <c r="I30">
         <f t="shared" si="1"/>
-        <v>12436.219738648</v>
+        <v>12786.885620647998</v>
       </c>
       <c r="J30">
         <f t="shared" si="2"/>
-        <v>12.436219738648001</v>
+        <v>12.786885620647997</v>
       </c>
       <c r="L30" s="1">
         <f t="shared" si="3"/>
-        <v>77.631106581344241</v>
+        <v>75.50216124879006</v>
       </c>
       <c r="M30" s="1">
         <f t="shared" si="4"/>
-        <v>9.8847892995950097</v>
+        <v>12.356097073776224</v>
       </c>
       <c r="N30" s="1">
         <f t="shared" si="5"/>
-        <v>3.0151364954955731</v>
+        <v>2.9324497858533105</v>
       </c>
       <c r="O30" s="1">
         <f t="shared" si="6"/>
-        <v>2.425866309377368E-2</v>
+        <v>2.3593396683930887E-2</v>
       </c>
       <c r="P30" s="1">
         <f t="shared" si="7"/>
-        <v>6.7436569763536056E-2</v>
+        <v>6.5587198077830283E-2</v>
       </c>
       <c r="Q30" s="1">
         <f t="shared" si="8"/>
-        <v>6.2586140833550159</v>
+        <v>6.0869786677622333</v>
       </c>
       <c r="R30" s="1">
         <f t="shared" si="9"/>
-        <v>3.118658307352844</v>
+        <v>3.0331326290564364</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.35">
@@ -14209,7 +14215,7 @@
         <v>10176.9</v>
       </c>
       <c r="C31">
-        <v>1215</v>
+        <v>1579.96</v>
       </c>
       <c r="D31">
         <v>365.65300000000002</v>
@@ -14228,39 +14234,39 @@
       </c>
       <c r="I31">
         <f t="shared" si="1"/>
-        <v>12907.136424315999</v>
+        <v>13272.096424316</v>
       </c>
       <c r="J31">
         <f t="shared" si="2"/>
-        <v>12.907136424315999</v>
+        <v>13.272096424316</v>
       </c>
       <c r="L31" s="1">
         <f t="shared" si="3"/>
-        <v>78.847078588458587</v>
+        <v>76.678918496664579</v>
       </c>
       <c r="M31" s="1">
         <f t="shared" si="4"/>
-        <v>9.4133970546018126</v>
+        <v>11.904374030204696</v>
       </c>
       <c r="N31" s="1">
         <f t="shared" si="5"/>
-        <v>2.8329521590175446</v>
+        <v>2.755050809682801</v>
       </c>
       <c r="O31" s="1">
         <f t="shared" si="6"/>
-        <v>2.0571443802188748E-2</v>
+        <v>2.0005764207193362E-2</v>
       </c>
       <c r="P31" s="1">
         <f t="shared" si="7"/>
-        <v>6.5531499179518712E-2</v>
+        <v>6.3729494795588856E-2</v>
       </c>
       <c r="Q31" s="1">
         <f t="shared" si="8"/>
-        <v>5.857573478309817</v>
+        <v>5.6965002048571547</v>
       </c>
       <c r="R31" s="1">
         <f t="shared" si="9"/>
-        <v>2.9628957766305337</v>
+        <v>2.8814211995879839</v>
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.35">
@@ -14271,7 +14277,7 @@
         <v>10240.36875</v>
       </c>
       <c r="C32">
-        <v>1200.705882</v>
+        <v>1579.96</v>
       </c>
       <c r="D32">
         <v>359.83049999999997</v>
@@ -14290,39 +14296,39 @@
       </c>
       <c r="I32">
         <f t="shared" si="1"/>
-        <v>12909.327184104999</v>
+        <v>13288.581302105</v>
       </c>
       <c r="J32">
         <f t="shared" si="2"/>
-        <v>12.909327184104999</v>
+        <v>13.288581302104999</v>
       </c>
       <c r="L32" s="1">
         <f t="shared" si="3"/>
-        <v>79.325348284678725</v>
+        <v>77.061414737913807</v>
       </c>
       <c r="M32" s="1">
         <f t="shared" si="4"/>
-        <v>9.3010725104125136</v>
+        <v>11.889606302440455</v>
       </c>
       <c r="N32" s="1">
         <f t="shared" si="5"/>
-        <v>2.7873683490108778</v>
+        <v>2.7078172742413096</v>
       </c>
       <c r="O32" s="1">
         <f t="shared" si="6"/>
-        <v>1.8072504776799093E-2</v>
+        <v>1.75567182000868E-2</v>
       </c>
       <c r="P32" s="1">
         <f t="shared" si="7"/>
-        <v>6.348443428632633E-2</v>
+        <v>6.1672598050040085E-2</v>
       </c>
       <c r="Q32" s="1">
         <f t="shared" si="8"/>
-        <v>5.5806703922342882</v>
+        <v>5.4213988959519668</v>
       </c>
       <c r="R32" s="1">
         <f t="shared" si="9"/>
-        <v>2.9239835246004704</v>
+        <v>2.8405334732023411</v>
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.35">
@@ -14333,7 +14339,7 @@
         <v>10303.75</v>
       </c>
       <c r="C33">
-        <v>1191.176471</v>
+        <v>1579.96</v>
       </c>
       <c r="D33">
         <v>354.00799999999998</v>
@@ -14352,39 +14358,39 @@
       </c>
       <c r="I33">
         <f t="shared" si="1"/>
-        <v>12913.435262141002</v>
+        <v>13302.218791141</v>
       </c>
       <c r="J33">
         <f t="shared" si="2"/>
-        <v>12.913435262141002</v>
+        <v>13.302218791141</v>
       </c>
       <c r="L33" s="1">
         <f t="shared" si="3"/>
-        <v>79.790929298325807</v>
+        <v>77.458882324669645</v>
       </c>
       <c r="M33" s="1">
         <f t="shared" si="4"/>
-        <v>9.224319066300156</v>
+        <v>11.877417029497519</v>
       </c>
       <c r="N33" s="1">
         <f t="shared" si="5"/>
-        <v>2.7413929199603753</v>
+        <v>2.661270315563911</v>
       </c>
       <c r="O33" s="1">
         <f t="shared" si="6"/>
-        <v>1.6856380427148279E-2</v>
+        <v>1.6363719528126104E-2</v>
       </c>
       <c r="P33" s="1">
         <f t="shared" si="7"/>
-        <v>6.1428942074432988E-2</v>
+        <v>5.9633560322154194E-2</v>
       </c>
       <c r="Q33" s="1">
         <f t="shared" si="8"/>
-        <v>5.3594775723934944</v>
+        <v>5.2028362904459158</v>
       </c>
       <c r="R33" s="1">
         <f t="shared" si="9"/>
-        <v>2.8055958205185765</v>
+        <v>2.7235967599727307</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.35">
@@ -14395,7 +14401,7 @@
         <v>10440.35</v>
       </c>
       <c r="C34">
-        <v>1181.6470589999999</v>
+        <v>1579.96</v>
       </c>
       <c r="D34">
         <v>348.57366669999999</v>
@@ -14414,39 +14420,39 @@
       </c>
       <c r="I34">
         <f t="shared" si="1"/>
-        <v>13006.630094876002</v>
+        <v>13404.943035876002</v>
       </c>
       <c r="J34">
         <f t="shared" si="2"/>
-        <v>13.006630094876002</v>
+        <v>13.404943035876002</v>
       </c>
       <c r="L34" s="1">
         <f t="shared" si="3"/>
-        <v>80.269446611793825</v>
+        <v>77.884329475016912</v>
       </c>
       <c r="M34" s="1">
         <f t="shared" si="4"/>
-        <v>9.0849593659583903</v>
+        <v>11.786398463398998</v>
       </c>
       <c r="N34" s="1">
         <f t="shared" si="5"/>
-        <v>2.6799690938955938</v>
+        <v>2.6003367993963353</v>
       </c>
       <c r="O34" s="1">
         <f t="shared" si="6"/>
-        <v>1.5903925620325877E-2</v>
+        <v>1.5431358197225053E-2</v>
       </c>
       <c r="P34" s="1">
         <f t="shared" si="7"/>
-        <v>5.8968079695151193E-2</v>
+        <v>5.7215908933542052E-2</v>
       </c>
       <c r="Q34" s="1">
         <f t="shared" si="8"/>
-        <v>5.2302410857982151</v>
+        <v>5.074830301623467</v>
       </c>
       <c r="R34" s="1">
         <f t="shared" si="9"/>
-        <v>2.6605118372384911</v>
+        <v>2.5814576934335061</v>
       </c>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.35">
@@ -14457,7 +14463,7 @@
         <v>10571.35</v>
       </c>
       <c r="C35">
-        <v>1172.117647</v>
+        <v>1579.96</v>
       </c>
       <c r="D35">
         <v>343.13933329999998</v>
@@ -14476,39 +14482,39 @@
       </c>
       <c r="I35">
         <f t="shared" si="1"/>
-        <v>13094.170480269</v>
+        <v>13502.012833269</v>
       </c>
       <c r="J35">
         <f t="shared" si="2"/>
-        <v>13.094170480269</v>
+        <v>13.502012833268999</v>
       </c>
       <c r="L35" s="1">
         <f t="shared" ref="L35:L57" si="10">B35/$I35*100</f>
-        <v>80.73325466419945</v>
+        <v>78.294622665090074</v>
       </c>
       <c r="M35" s="1">
         <f t="shared" si="4"/>
-        <v>8.9514463613117758</v>
+        <v>11.701662704000501</v>
       </c>
       <c r="N35" s="1">
         <f t="shared" si="5"/>
-        <v>2.6205503725269255</v>
+        <v>2.5413939205753353</v>
       </c>
       <c r="O35" s="1">
         <f t="shared" si="6"/>
-        <v>1.5002961088373139E-2</v>
+        <v>1.4549781030865513E-2</v>
       </c>
       <c r="P35" s="1">
         <f t="shared" si="7"/>
-        <v>5.6475411543962739E-2</v>
+        <v>5.4769512948311908E-2</v>
       </c>
       <c r="Q35" s="1">
         <f t="shared" si="8"/>
-        <v>5.104052481270811</v>
+        <v>4.9498792628401649</v>
       </c>
       <c r="R35" s="1">
         <f t="shared" si="9"/>
-        <v>2.5192177480587019</v>
+        <v>2.4431221535147536</v>
       </c>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.35">
@@ -14519,7 +14525,7 @@
         <v>10553.79722</v>
       </c>
       <c r="C36">
-        <v>1162.5882349999999</v>
+        <v>1579.96</v>
       </c>
       <c r="D36">
         <v>337.70499999999998</v>
@@ -14538,39 +14544,39 @@
       </c>
       <c r="I36">
         <f t="shared" si="1"/>
-        <v>13045.343956037001</v>
+        <v>13462.715721037001</v>
       </c>
       <c r="J36">
         <f t="shared" si="2"/>
-        <v>13.045343956037001</v>
+        <v>13.462715721037</v>
       </c>
       <c r="L36" s="1">
         <f t="shared" si="10"/>
-        <v>80.90087356505471</v>
+        <v>78.39278076345704</v>
       </c>
       <c r="M36" s="1">
         <f t="shared" si="4"/>
-        <v>8.9119017399459857</v>
+        <v>11.735819375069591</v>
       </c>
       <c r="N36" s="1">
         <f t="shared" si="5"/>
-        <v>2.588701387545401</v>
+        <v>2.5084463417161675</v>
       </c>
       <c r="O36" s="1">
         <f t="shared" si="6"/>
-        <v>1.4111965236056966E-2</v>
+        <v>1.3674465406138696E-2</v>
       </c>
       <c r="P36" s="1">
         <f t="shared" si="7"/>
-        <v>5.4580495209595264E-2</v>
+        <v>5.2888388052893892E-2</v>
       </c>
       <c r="Q36" s="1">
         <f t="shared" si="8"/>
-        <v>5.1374447125240605</v>
+        <v>4.9781734026570996</v>
       </c>
       <c r="R36" s="1">
         <f t="shared" si="9"/>
-        <v>2.3923861344841866</v>
+        <v>2.3182172636410696</v>
       </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.35">
@@ -14581,7 +14587,7 @@
         <v>10535.85556</v>
       </c>
       <c r="C37">
-        <v>1153.058824</v>
+        <v>1579.96</v>
       </c>
       <c r="D37">
         <v>335.37599999999998</v>
@@ -14600,39 +14606,39 @@
       </c>
       <c r="I37">
         <f t="shared" si="1"/>
-        <v>12999.479141269001</v>
+        <v>13426.380317269</v>
       </c>
       <c r="J37">
         <f t="shared" si="2"/>
-        <v>12.999479141269001</v>
+        <v>13.426380317269</v>
       </c>
       <c r="L37" s="1">
         <f t="shared" si="10"/>
-        <v>81.048290054577492</v>
+        <v>78.471302845851838</v>
       </c>
       <c r="M37" s="1">
         <f t="shared" si="4"/>
-        <v>8.8700386490057408</v>
+        <v>11.767579665294127</v>
       </c>
       <c r="N37" s="1">
         <f t="shared" si="5"/>
-        <v>2.5799187517851641</v>
+        <v>2.497888426180209</v>
       </c>
       <c r="O37" s="1">
         <f t="shared" si="6"/>
-        <v>1.3135446047058397E-2</v>
+        <v>1.2717795330166266E-2</v>
       </c>
       <c r="P37" s="1">
         <f t="shared" si="7"/>
-        <v>5.2659340621333178E-2</v>
+        <v>5.0984999964550387E-2</v>
       </c>
       <c r="Q37" s="1">
         <f t="shared" si="8"/>
-        <v>5.1674480646493421</v>
+        <v>5.0031454303138334</v>
       </c>
       <c r="R37" s="1">
         <f t="shared" si="9"/>
-        <v>2.2685096933138551</v>
+        <v>2.1963808370652735</v>
       </c>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.35">
@@ -14643,7 +14649,7 @@
         <v>10517.525</v>
       </c>
       <c r="C38">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D38">
         <v>333.04700000000003</v>
@@ -14662,39 +14668,39 @@
       </c>
       <c r="I38">
         <f t="shared" si="1"/>
-        <v>12953.541977141</v>
+        <v>13389.972565141001</v>
       </c>
       <c r="J38">
         <f t="shared" si="2"/>
-        <v>12.953541977141001</v>
+        <v>13.389972565141001</v>
       </c>
       <c r="L38" s="1">
         <f t="shared" si="10"/>
-        <v>81.194201698347698</v>
+        <v>78.547771093877856</v>
       </c>
       <c r="M38" s="1">
         <f t="shared" si="4"/>
-        <v>8.8279284076739497</v>
+        <v>11.799576080635251</v>
       </c>
       <c r="N38" s="1">
         <f t="shared" si="5"/>
-        <v>2.5710882829401029</v>
+        <v>2.4872866496160215</v>
       </c>
       <c r="O38" s="1">
         <f t="shared" si="6"/>
-        <v>1.218296234176647E-2</v>
+        <v>1.1785872848675114E-2</v>
       </c>
       <c r="P38" s="1">
         <f t="shared" si="7"/>
-        <v>5.2846086515024898E-2</v>
+        <v>5.112362976621166E-2</v>
       </c>
       <c r="Q38" s="1">
         <f t="shared" si="8"/>
-        <v>5.1976929127812355</v>
+        <v>5.0282801553515366</v>
       </c>
       <c r="R38" s="1">
         <f t="shared" si="9"/>
-        <v>2.1440596494002229</v>
+        <v>2.0741765179044291</v>
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.35">
@@ -14705,7 +14711,7 @@
         <v>10455.82778</v>
       </c>
       <c r="C39">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D39">
         <v>333.04700000000003</v>
@@ -14724,39 +14730,39 @@
       </c>
       <c r="I39">
         <f t="shared" si="1"/>
-        <v>12891.844757141</v>
+        <v>13328.275345140999</v>
       </c>
       <c r="J39">
         <f t="shared" si="2"/>
-        <v>12.891844757141</v>
+        <v>13.328275345140998</v>
       </c>
       <c r="L39" s="1">
         <f t="shared" si="10"/>
-        <v>81.104201741246911</v>
+        <v>78.448467706752552</v>
       </c>
       <c r="M39" s="1">
         <f t="shared" si="4"/>
-        <v>8.870176716692006</v>
+        <v>11.854196879088303</v>
       </c>
       <c r="N39" s="1">
         <f t="shared" si="5"/>
-        <v>2.5833928834391213</v>
+        <v>2.4988004177255894</v>
       </c>
       <c r="O39" s="1">
         <f t="shared" si="6"/>
-        <v>1.2241267023680618E-2</v>
+        <v>1.1840430214216173E-2</v>
       </c>
       <c r="P39" s="1">
         <f t="shared" si="7"/>
-        <v>5.3098994976713478E-2</v>
+        <v>5.136028347805402E-2</v>
       </c>
       <c r="Q39" s="1">
         <f t="shared" si="8"/>
-        <v>5.2225678014549199</v>
+        <v>5.0515563031600728</v>
       </c>
       <c r="R39" s="1">
         <f t="shared" si="9"/>
-        <v>2.1543205951666455</v>
+        <v>2.0837779795812126</v>
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.35">
@@ -14767,7 +14773,7 @@
         <v>10393.936110000001</v>
       </c>
       <c r="C40">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D40">
         <v>333.04700000000003</v>
@@ -14786,39 +14792,39 @@
       </c>
       <c r="I40">
         <f t="shared" si="1"/>
-        <v>12829.953087141001</v>
+        <v>13266.383675141002</v>
       </c>
       <c r="J40">
         <f t="shared" si="2"/>
-        <v>12.829953087141</v>
+        <v>13.266383675141002</v>
       </c>
       <c r="L40" s="1">
         <f t="shared" si="10"/>
-        <v>81.013048445340516</v>
+        <v>78.347923326509161</v>
       </c>
       <c r="M40" s="1">
         <f t="shared" si="4"/>
-        <v>8.9129664327932616</v>
+        <v>11.909500272938605</v>
       </c>
       <c r="N40" s="1">
         <f t="shared" si="5"/>
-        <v>2.5958551659382221</v>
+        <v>2.5104580732432362</v>
       </c>
       <c r="O40" s="1">
         <f t="shared" si="6"/>
-        <v>1.230031887319758E-2</v>
+        <v>1.1895669382434221E-2</v>
       </c>
       <c r="P40" s="1">
         <f t="shared" si="7"/>
-        <v>5.3355144430426153E-2</v>
+        <v>5.1599894648209348E-2</v>
       </c>
       <c r="Q40" s="1">
         <f t="shared" si="8"/>
-        <v>5.2477614588849093</v>
+        <v>5.0751233326805165</v>
       </c>
       <c r="R40" s="1">
         <f t="shared" si="9"/>
-        <v>2.1647130337394644</v>
+        <v>2.0934994305978276</v>
       </c>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.35">
@@ -14829,7 +14835,7 @@
         <v>10331.85</v>
       </c>
       <c r="C41">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D41">
         <v>333.04700000000003</v>
@@ -14848,39 +14854,39 @@
       </c>
       <c r="I41">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J41">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L41" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M41" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N41" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O41" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P41" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q41" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R41" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.35">
@@ -14891,7 +14897,7 @@
         <v>10331.85</v>
       </c>
       <c r="C42">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D42">
         <v>333.04700000000003</v>
@@ -14910,39 +14916,39 @@
       </c>
       <c r="I42">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J42">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L42" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M42" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N42" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O42" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P42" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q42" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R42" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.35">
@@ -14953,7 +14959,7 @@
         <v>10331.85</v>
       </c>
       <c r="C43">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D43">
         <v>333.04700000000003</v>
@@ -14972,39 +14978,39 @@
       </c>
       <c r="I43">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J43">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L43" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M43" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N43" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O43" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P43" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q43" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R43" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.35">
@@ -15015,7 +15021,7 @@
         <v>10331.85</v>
       </c>
       <c r="C44">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D44">
         <v>333.04700000000003</v>
@@ -15034,39 +15040,39 @@
       </c>
       <c r="I44">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J44">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L44" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M44" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N44" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O44" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P44" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q44" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R44" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.35">
@@ -15077,7 +15083,7 @@
         <v>10331.85</v>
       </c>
       <c r="C45">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D45">
         <v>333.04700000000003</v>
@@ -15096,39 +15102,39 @@
       </c>
       <c r="I45">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J45">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L45" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M45" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N45" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O45" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P45" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q45" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R45" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.35">
@@ -15139,7 +15145,7 @@
         <v>10331.85</v>
       </c>
       <c r="C46">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D46">
         <v>333.04700000000003</v>
@@ -15158,39 +15164,39 @@
       </c>
       <c r="I46">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J46">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L46" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M46" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N46" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O46" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P46" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q46" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R46" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.35">
@@ -15201,7 +15207,7 @@
         <v>10331.85</v>
       </c>
       <c r="C47">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D47">
         <v>333.04700000000003</v>
@@ -15220,39 +15226,39 @@
       </c>
       <c r="I47">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J47">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L47" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M47" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N47" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O47" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P47" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q47" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R47" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.35">
@@ -15263,7 +15269,7 @@
         <v>10331.85</v>
       </c>
       <c r="C48">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D48">
         <v>333.04700000000003</v>
@@ -15282,39 +15288,39 @@
       </c>
       <c r="I48">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J48">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L48" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M48" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N48" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O48" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P48" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q48" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R48" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.35">
@@ -15325,7 +15331,7 @@
         <v>10331.85</v>
       </c>
       <c r="C49">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D49">
         <v>333.04700000000003</v>
@@ -15344,39 +15350,39 @@
       </c>
       <c r="I49">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J49">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L49" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M49" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N49" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O49" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P49" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q49" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R49" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.35">
@@ -15387,7 +15393,7 @@
         <v>10331.85</v>
       </c>
       <c r="C50">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D50">
         <v>333.04700000000003</v>
@@ -15406,39 +15412,39 @@
       </c>
       <c r="I50">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J50">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L50" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M50" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N50" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O50" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P50" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q50" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R50" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
     <row r="51" spans="1:18" x14ac:dyDescent="0.35">
@@ -15449,7 +15455,7 @@
         <v>10331.85</v>
       </c>
       <c r="C51">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D51">
         <v>333.04700000000003</v>
@@ -15468,39 +15474,39 @@
       </c>
       <c r="I51">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J51">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L51" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M51" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N51" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O51" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P51" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q51" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R51" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
     <row r="52" spans="1:18" x14ac:dyDescent="0.35">
@@ -15511,7 +15517,7 @@
         <v>10331.85</v>
       </c>
       <c r="C52">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D52">
         <v>333.04700000000003</v>
@@ -15530,39 +15536,39 @@
       </c>
       <c r="I52">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J52">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L52" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M52" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N52" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O52" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P52" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q52" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R52" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
     <row r="53" spans="1:18" x14ac:dyDescent="0.35">
@@ -15573,7 +15579,7 @@
         <v>10331.85</v>
       </c>
       <c r="C53">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D53">
         <v>333.04700000000003</v>
@@ -15592,39 +15598,39 @@
       </c>
       <c r="I53">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J53">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L53" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M53" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N53" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O53" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P53" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q53" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R53" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
     <row r="54" spans="1:18" x14ac:dyDescent="0.35">
@@ -15635,7 +15641,7 @@
         <v>10331.85</v>
       </c>
       <c r="C54">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D54">
         <v>333.04700000000003</v>
@@ -15654,39 +15660,39 @@
       </c>
       <c r="I54">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J54">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L54" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M54" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N54" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O54" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P54" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q54" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R54" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
     <row r="55" spans="1:18" x14ac:dyDescent="0.35">
@@ -15697,7 +15703,7 @@
         <v>10331.85</v>
       </c>
       <c r="C55">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D55">
         <v>333.04700000000003</v>
@@ -15716,39 +15722,39 @@
       </c>
       <c r="I55">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J55">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L55" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M55" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N55" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O55" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P55" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q55" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R55" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
     <row r="56" spans="1:18" x14ac:dyDescent="0.35">
@@ -15759,7 +15765,7 @@
         <v>10331.85</v>
       </c>
       <c r="C56">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D56">
         <v>333.04700000000003</v>
@@ -15778,39 +15784,39 @@
       </c>
       <c r="I56">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J56">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L56" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M56" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N56" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O56" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P56" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q56" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R56" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
     <row r="57" spans="1:18" x14ac:dyDescent="0.35">
@@ -15821,7 +15827,7 @@
         <v>10331.85</v>
       </c>
       <c r="C57">
-        <v>1143.5294120000001</v>
+        <v>1579.96</v>
       </c>
       <c r="D57">
         <v>333.04700000000003</v>
@@ -15840,39 +15846,39 @@
       </c>
       <c r="I57">
         <f t="shared" si="1"/>
-        <v>12767.866977141</v>
+        <v>13204.297565141002</v>
       </c>
       <c r="J57">
         <f t="shared" si="2"/>
-        <v>12.767866977141001</v>
+        <v>13.204297565141001</v>
       </c>
       <c r="L57" s="1">
         <f t="shared" si="10"/>
-        <v>80.920720888600002</v>
+        <v>78.246116077206665</v>
       </c>
       <c r="M57" s="1">
         <f t="shared" si="4"/>
-        <v>8.9563073773193462</v>
+        <v>11.965498294820717</v>
       </c>
       <c r="N57" s="1">
         <f t="shared" si="5"/>
-        <v>2.6084779908521289</v>
+        <v>2.5222621525830755</v>
       </c>
       <c r="O57" s="1">
         <f t="shared" si="6"/>
-        <v>1.2360131444237336E-2</v>
+        <v>1.1951602371989925E-2</v>
       </c>
       <c r="P57" s="1">
         <f t="shared" si="7"/>
-        <v>5.3614593669058117E-2</v>
+        <v>5.1842515410072107E-2</v>
       </c>
       <c r="Q57" s="1">
         <f t="shared" si="8"/>
-        <v>5.2732796676642932</v>
+        <v>5.0989863715087402</v>
       </c>
       <c r="R57" s="1">
         <f t="shared" si="9"/>
-        <v>2.1752393504509246</v>
+        <v>2.10334298609874</v>
       </c>
     </row>
   </sheetData>

</xml_diff>